<commit_message>
Job-search reporting refresh: charts, workbook, presentation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/my-data.xlsx
+++ b/my-data.xlsx
@@ -435,7 +435,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Built by build_presentation.py from the PostgreSQL reporting views after each pipeline snapshot (snapshot 2026-10-25). Fit rates are shares of the shortlist the AI judge graded, not of every posting.</t>
+          <t>Built by build_presentation.py from the PostgreSQL reporting views after each pipeline snapshot (snapshot 2026-10-28). Fit rates are shares of the shortlist the AI judge graded, not of every posting.</t>
         </is>
       </c>
     </row>
@@ -445,14 +445,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Slide 1: Technology &amp; telecom good-fit rate 26% = Industry!C6; share of postings (about a third) = Industry!B6.</t>
+          <t>Slide 1: Technology &amp; telecom good-fit rate 25% = Industry!C5; share of postings (about a third) = Industry!B5.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Slide 4: remote 45.0% = Workplace!B2.</t>
+          <t>Slide 4: remote 44.1% = Workplace!B2.</t>
         </is>
       </c>
     </row>
@@ -529,26 +529,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15.1</v>
+        <v>14.8</v>
       </c>
       <c r="C2" t="n">
-        <v>45.5</v>
+        <v>47.4</v>
       </c>
       <c r="D2" t="n">
-        <v>60.4</v>
+        <v>63.4</v>
       </c>
       <c r="E2" t="n">
-        <v>17.6</v>
+        <v>19.7</v>
       </c>
       <c r="F2" t="n">
-        <v>12.6</v>
+        <v>14.7</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -559,116 +559,116 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14.3</v>
+        <v>14.1</v>
       </c>
       <c r="C3" t="n">
-        <v>44.8</v>
+        <v>46.2</v>
       </c>
       <c r="D3" t="n">
-        <v>51.4</v>
+        <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>21.9</v>
+        <v>20.2</v>
       </c>
       <c r="F3" t="n">
-        <v>14.1</v>
+        <v>14.8</v>
       </c>
       <c r="G3" t="n">
         <v>18.2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Government &amp; defense</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.3</v>
+        <v>11.1</v>
       </c>
       <c r="C4" t="n">
-        <v>33.3</v>
+        <v>28.3</v>
       </c>
       <c r="D4" t="n">
-        <v>33.3</v>
+        <v>44.9</v>
       </c>
       <c r="E4" t="n">
-        <v>33.3</v>
+        <v>22.4</v>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>6.1</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Government &amp; defense</t>
+          <t>Technology &amp; telecom</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11.8</v>
+        <v>34.2</v>
       </c>
       <c r="C5" t="n">
-        <v>32.3</v>
+        <v>25.3</v>
       </c>
       <c r="D5" t="n">
-        <v>47.4</v>
+        <v>33.7</v>
       </c>
       <c r="E5" t="n">
-        <v>21.1</v>
+        <v>17.8</v>
       </c>
       <c r="F5" t="n">
-        <v>8.800000000000001</v>
+        <v>13.2</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Technology &amp; telecom</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33</v>
+        <v>2.1</v>
       </c>
       <c r="C6" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D6" t="n">
-        <v>40.3</v>
+        <v>33.3</v>
       </c>
       <c r="E6" t="n">
-        <v>16.7</v>
+        <v>33.3</v>
       </c>
       <c r="F6" t="n">
-        <v>12.6</v>
+        <v>20</v>
       </c>
       <c r="G6" t="n">
-        <v>18.2</v>
+        <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -679,26 +679,26 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11.6</v>
+        <v>12.2</v>
       </c>
       <c r="C7" t="n">
-        <v>24.8</v>
+        <v>23.3</v>
       </c>
       <c r="D7" t="n">
-        <v>25</v>
+        <v>23.3</v>
       </c>
       <c r="E7" t="n">
         <v>25.8</v>
       </c>
       <c r="F7" t="n">
-        <v>10.9</v>
+        <v>10.1</v>
       </c>
       <c r="G7" t="n">
         <v>54.5</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-25</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -780,11 +780,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45</v>
+        <v>44.1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-25</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -795,11 +795,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>42.7</v>
+        <v>44.7</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-25</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -810,11 +810,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10.6</v>
+        <v>9</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-25</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -825,11 +825,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-25</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Job-search reporting refresh: presentation and charts (auto, snapshot 2026-10-28 16:07:42.243331-04)
</commit_message>
<xml_diff>
--- a/my-data.xlsx
+++ b/my-data.xlsx
@@ -445,14 +445,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Slide 1: Technology &amp; telecom good-fit rate 25% = Industry!C5; share of postings (about a third) = Industry!B5.</t>
+          <t>Slide 1: Technology &amp; telecom good-fit rate 26% = Industry!C5; share of postings (about a third) = Industry!B5.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Slide 4: remote 44.1% = Workplace!B2.</t>
+          <t>Slide 4: remote 44.2% = Workplace!B2.</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
         <v>14.1</v>
       </c>
       <c r="C3" t="n">
-        <v>46.2</v>
+        <v>46.7</v>
       </c>
       <c r="D3" t="n">
         <v>50</v>
@@ -622,7 +622,7 @@
         <v>34.2</v>
       </c>
       <c r="C5" t="n">
-        <v>25.3</v>
+        <v>25.7</v>
       </c>
       <c r="D5" t="n">
         <v>33.7</v>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44.1</v>
+        <v>44.2</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Job-search reporting refresh: presentation and charts (auto, snapshot 2026-10-29 03:21:25.137592-04)
</commit_message>
<xml_diff>
--- a/my-data.xlsx
+++ b/my-data.xlsx
@@ -435,7 +435,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Built by build_presentation.py from the PostgreSQL reporting views after each pipeline snapshot (snapshot 2026-10-28). Fit rates are shares of the shortlist the AI judge graded, not of every posting.</t>
+          <t>Built by build_presentation.py from the PostgreSQL reporting views after each pipeline snapshot (snapshot 2026-10-29). Fit rates are shares of the shortlist the AI judge graded, not of every posting.</t>
         </is>
       </c>
     </row>
@@ -452,7 +452,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Slide 4: remote 44.2% = Workplace!B2.</t>
+          <t>Slide 4: remote 43.0% = Workplace!B2.</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -529,26 +529,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14.8</v>
+        <v>15.1</v>
       </c>
       <c r="C2" t="n">
-        <v>47.4</v>
+        <v>48</v>
       </c>
       <c r="D2" t="n">
-        <v>63.4</v>
+        <v>63.8</v>
       </c>
       <c r="E2" t="n">
-        <v>19.7</v>
+        <v>18.8</v>
       </c>
       <c r="F2" t="n">
-        <v>14.7</v>
+        <v>16.7</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -559,56 +559,56 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F3" t="n">
         <v>14.1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="D3" t="n">
-        <v>50</v>
-      </c>
-      <c r="E3" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="F3" t="n">
-        <v>14.8</v>
       </c>
       <c r="G3" t="n">
         <v>18.2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Government &amp; defense</t>
+          <t>Insurance</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11.1</v>
+        <v>2.4</v>
       </c>
       <c r="C4" t="n">
-        <v>28.3</v>
+        <v>26.7</v>
       </c>
       <c r="D4" t="n">
-        <v>44.9</v>
+        <v>28.6</v>
       </c>
       <c r="E4" t="n">
-        <v>22.4</v>
+        <v>35.7</v>
       </c>
       <c r="F4" t="n">
-        <v>6.1</v>
+        <v>21.4</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -619,56 +619,56 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D5" t="n">
         <v>34.2</v>
       </c>
-      <c r="C5" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="D5" t="n">
-        <v>33.7</v>
-      </c>
       <c r="E5" t="n">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="F5" t="n">
-        <v>13.2</v>
+        <v>12.6</v>
       </c>
       <c r="G5" t="n">
         <v>18.2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Government &amp; defense</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.1</v>
+        <v>11</v>
       </c>
       <c r="C6" t="n">
         <v>25</v>
       </c>
       <c r="D6" t="n">
-        <v>33.3</v>
+        <v>44.4</v>
       </c>
       <c r="E6" t="n">
-        <v>33.3</v>
+        <v>22.2</v>
       </c>
       <c r="F6" t="n">
-        <v>20</v>
+        <v>6.7</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -679,56 +679,26 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12.2</v>
+        <v>12.7</v>
       </c>
       <c r="C7" t="n">
-        <v>23.3</v>
+        <v>22.7</v>
       </c>
       <c r="D7" t="n">
-        <v>23.3</v>
+        <v>22.5</v>
       </c>
       <c r="E7" t="n">
         <v>25.8</v>
       </c>
       <c r="F7" t="n">
-        <v>10.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G7" t="n">
         <v>54.5</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Retail, travel &amp; consumer</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="C8" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="D8" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="E8" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-28</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -780,11 +750,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44.2</v>
+        <v>43</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -795,11 +765,11 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>44.7</v>
+        <v>45.3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -810,11 +780,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8.9</v>
+        <v>9.5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -825,11 +795,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-28</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Job-search reporting refresh: presentation and charts (auto, snapshot 2026-10-29 09:41:05.187705-04)
</commit_message>
<xml_diff>
--- a/my-data.xlsx
+++ b/my-data.xlsx
@@ -452,7 +452,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Slide 4: remote 43.0% = Workplace!B2.</t>
+          <t>Slide 4: remote 43.3% = Workplace!B2.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
         <v>33.5</v>
       </c>
       <c r="C5" t="n">
-        <v>25.9</v>
+        <v>26.3</v>
       </c>
       <c r="D5" t="n">
         <v>34.2</v>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>43</v>
+        <v>43.3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45.3</v>
+        <v>45</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -780,7 +780,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.5</v>
+        <v>9.4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Job-search reporting refresh: presentation and charts (auto, snapshot 2026-10-30 15:14:43.460762-04)
</commit_message>
<xml_diff>
--- a/my-data.xlsx
+++ b/my-data.xlsx
@@ -435,7 +435,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Built by build_presentation.py from the PostgreSQL reporting views after each pipeline snapshot (snapshot 2026-10-29). Fit rates are shares of the shortlist the AI judge graded, not of every posting.</t>
+          <t>Built by build_presentation.py from the PostgreSQL reporting views after each pipeline snapshot (snapshot 2026-10-30). Fit rates are shares of the shortlist the AI judge graded, not of every posting.</t>
         </is>
       </c>
     </row>
@@ -445,14 +445,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Slide 1: Technology &amp; telecom good-fit rate 26% = Industry!C5; share of postings (about a third) = Industry!B5.</t>
+          <t>Slide 1: Technology &amp; telecom good-fit rate 26% = Industry!C4; share of postings (about a third) = Industry!B4.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Slide 4: remote 43.3% = Workplace!B2.</t>
+          <t>Slide 4: remote 45.0% = Workplace!B2.</t>
         </is>
       </c>
     </row>
@@ -529,26 +529,26 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15.1</v>
+        <v>15.4</v>
       </c>
       <c r="C2" t="n">
-        <v>48</v>
+        <v>49.3</v>
       </c>
       <c r="D2" t="n">
-        <v>63.8</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>18.8</v>
+        <v>20.3</v>
       </c>
       <c r="F2" t="n">
-        <v>16.7</v>
+        <v>18</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14.2</v>
+        <v>13.7</v>
       </c>
       <c r="C3" t="n">
-        <v>46.1</v>
+        <v>44.2</v>
       </c>
       <c r="D3" t="n">
-        <v>50.5</v>
+        <v>50</v>
       </c>
       <c r="E3" t="n">
-        <v>19.8</v>
+        <v>20.2</v>
       </c>
       <c r="F3" t="n">
         <v>14.1</v>
@@ -578,67 +578,67 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Technology &amp; telecom</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.4</v>
+        <v>33.8</v>
       </c>
       <c r="C4" t="n">
-        <v>26.7</v>
+        <v>25.6</v>
       </c>
       <c r="D4" t="n">
-        <v>28.6</v>
+        <v>34.2</v>
       </c>
       <c r="E4" t="n">
-        <v>35.7</v>
+        <v>17.1</v>
       </c>
       <c r="F4" t="n">
-        <v>21.4</v>
+        <v>12.2</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>18.2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Technology &amp; telecom</t>
+          <t>Financial services</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33.5</v>
+        <v>12.4</v>
       </c>
       <c r="C5" t="n">
-        <v>26.3</v>
+        <v>23.5</v>
       </c>
       <c r="D5" t="n">
-        <v>34.2</v>
+        <v>23.4</v>
       </c>
       <c r="E5" t="n">
-        <v>17.4</v>
+        <v>27</v>
       </c>
       <c r="F5" t="n">
-        <v>12.6</v>
+        <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>18.2</v>
+        <v>54.5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -649,56 +649,56 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="C6" t="n">
-        <v>25</v>
+        <v>22.9</v>
       </c>
       <c r="D6" t="n">
-        <v>44.4</v>
+        <v>41.3</v>
       </c>
       <c r="E6" t="n">
-        <v>22.2</v>
+        <v>21.7</v>
       </c>
       <c r="F6" t="n">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Financial services</t>
+          <t>Retail, travel &amp; consumer</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12.7</v>
+        <v>8.9</v>
       </c>
       <c r="C7" t="n">
-        <v>22.7</v>
+        <v>13.3</v>
       </c>
       <c r="D7" t="n">
-        <v>22.5</v>
+        <v>40</v>
       </c>
       <c r="E7" t="n">
-        <v>25.8</v>
+        <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>9.199999999999999</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>54.5</v>
+        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-29</t>
+          <t>reporting.fit_by_industry, lens_fit_by_industry; tracker history for screens; snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -750,11 +750,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>43.3</v>
+        <v>45</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -780,11 +780,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.4</v>
+        <v>7.6</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-30</t>
         </is>
       </c>
     </row>
@@ -795,11 +795,11 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>reporting.workplace_mix, snapshot 2026-10-29</t>
+          <t>reporting.workplace_mix, snapshot 2026-10-30</t>
         </is>
       </c>
     </row>

</xml_diff>